<commit_message>
Add Sales Tax rows to the buyers order template
- New "Tax Rate" input row (percent) and "Sales Tax" formula row, placed
  after Registration Fee and before Total Price
- Sales Tax = Trade Difference * Tax Rate; taxable base is the trade
  difference, noted in the cell comment and the README sheet
- Total Price now adds Sales Tax
- Leaving Tax Rate blank yields $0.00 tax, so the form still reproduces
  the source document exactly ($61,225.75)

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0163XvMSENuP7J3Nt4ti5Htq
</commit_message>
<xml_diff>
--- a/Buyers_Order_Worksheet_Template.xlsx
+++ b/Buyers_Order_Worksheet_Template.xlsx
@@ -12,7 +12,7 @@
     <sheet name="README (使い方・計算式)" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">'Buyers Order'!$A$1:$I$47</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">'Buyers Order'!$A$1:$I$49</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -90,14 +90,161 @@
         <r>
           <rPr>
             <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">州・郡市の合計税率を入力（例</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Total Price = Trade Difference + Doc Fee + Insp Fee + License/Title + Registration Fee</t>
+          <t xml:space="preserve">: 6.25% </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">なら </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">6.25% </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">または </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">0.0625</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">）。空欄なら税額 </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">0</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">。</t>
         </r>
       </text>
     </comment>
     <comment ref="H37" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Sales Tax = Trade Difference x Tax Rate
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">課税ベースを </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Trade Difference</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">（下取差額）としています。
+元の伝票にはない行です。</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Tax Rate </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">を空欄のままにすれば </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Sales Tax = $0.00 </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">となり、
+元の伝票と同じ結果になります。別ベースにする場合はこの式を書き換えてください。</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H38" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Total Price = Trade Difference + Doc Fee + Insp Fee + License/Title + Registration Fee + Sales Tax</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H39" authorId="0">
       <text>
         <r>
           <rPr>
@@ -134,7 +281,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H39" authorId="0">
+    <comment ref="H41" authorId="0">
       <text>
         <r>
           <rPr>
@@ -151,7 +298,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="95">
   <si>
     <t xml:space="preserve">Date:</t>
   </si>
@@ -259,6 +406,12 @@
   </si>
   <si>
     <t xml:space="preserve">Registration Fee:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tax Rate:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sales Tax:</t>
   </si>
   <si>
     <t xml:space="preserve">Total Price:</t>
@@ -818,10 +971,10 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">Total Price</t>
-  </si>
-  <si>
-    <t xml:space="preserve">= Trade Difference + Doc Fee + Insp Fee + License/Title + Registration Fee</t>
+    <t xml:space="preserve">Sales Tax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">= Trade Difference × Tax Rate</t>
   </si>
   <si>
     <r>
@@ -831,7 +984,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">例</t>
+      <t xml:space="preserve">課税ベースは </t>
     </r>
     <r>
       <rPr>
@@ -841,53 +994,8 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">: 60,484 + 225 + 123.75 + 271.75 + 121.25 = 61,225.75</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">Trade Payoff</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">= Trade In </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">欄の </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Payoff </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">を参照</t>
-    </r>
-  </si>
-  <si>
+      <t xml:space="preserve">Trade Difference</t>
+    </r>
     <r>
       <rPr>
         <sz val="9"/>
@@ -895,7 +1003,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">写真では両方 </t>
+      <t xml:space="preserve">（下取差額）。</t>
     </r>
     <r>
       <rPr>
@@ -905,7 +1013,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">$0.00</t>
+      <t xml:space="preserve">Tax Rate </t>
     </r>
     <r>
       <rPr>
@@ -914,38 +1022,33 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">。別値にする場合は上書き入力可（推定）。</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">Balance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">= Total Price + Trade Payoff − Deposit</t>
-  </si>
-  <si>
+      <t xml:space="preserve">を空欄にすれば </t>
+    </r>
     <r>
       <rPr>
         <sz val="9"/>
         <color rgb="FF666666"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">例</t>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">$0.00</t>
     </r>
     <r>
       <rPr>
         <sz val="9"/>
         <color rgb="FF666666"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">: 61,225.75 + 0.00 − 0.00 = 61,225.75</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">= Balance</t>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">。</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Price</t>
+  </si>
+  <si>
+    <t xml:space="preserve">= Trade Difference + Doc Fee + Insp Fee + License/Title + Registration Fee + Sales Tax</t>
   </si>
   <si>
     <r>
@@ -965,6 +1068,130 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
+      <t xml:space="preserve">: 60,484 + 225 + 123.75 + 271.75 + 121.25 + 0 = 61,225.75</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Trade Payoff</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">= Trade In </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">欄の </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Payoff </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">を参照</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">写真では両方 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">$0.00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">。別値にする場合は上書き入力可（推定）。</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Balance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">= Total Price + Trade Payoff − Deposit</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">例</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: 61,225.75 + 0.00 − 0.00 = 61,225.75</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">= Balance</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">例</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
       <t xml:space="preserve">: 61,225.75</t>
     </r>
   </si>
@@ -1055,26 +1282,134 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">税率</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(Sales Tax)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">の行は元の書式に存在しないため設けていません。必要なら追加します。</t>
+      <t xml:space="preserve">元の伝票にはない行ですが、あらかじめ用意してあります。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Tax Rate</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（黄色）に州・郡市の合計税率を入力すると自動計算され、</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Total Price </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">に加算されます。空欄のままなら税額 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">$0.00 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">で、元の伝票と完全に同じ結果になります。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">課税ベースは </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Trade Difference</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（下取差額）。州によって </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Total Purchase </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">基準の場合は </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Sales Tax </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">セルの式を書き換えてください。</t>
     </r>
   </si>
   <si>
@@ -1182,12 +1517,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
     <numFmt numFmtId="166" formatCode="\$#,##0.00;&quot;($&quot;#,##0.00\);\$0.00"/>
     <numFmt numFmtId="167" formatCode="#,##0"/>
     <numFmt numFmtId="168" formatCode="&quot;($&quot;#,##0.00\);&quot;($&quot;#,##0.00\);&quot;($0.00)&quot;"/>
+    <numFmt numFmtId="169" formatCode="0.000%"/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -1413,7 +1749,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1467,6 +1803,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="168" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1853,7 +2193,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
@@ -2076,7 +2416,7 @@
     </row>
     <row r="20" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="n">
-        <f aca="false">H39</f>
+        <f aca="false">H41</f>
         <v>0</v>
       </c>
       <c r="B20" s="11"/>
@@ -2214,11 +2554,8 @@
         <v>36</v>
       </c>
       <c r="G36" s="9"/>
-      <c r="H36" s="12" t="n">
-        <f aca="false">H30+H32+H33+H34+H35</f>
-        <v>0</v>
-      </c>
-      <c r="I36" s="12"/>
+      <c r="H36" s="14"/>
+      <c r="I36" s="14"/>
     </row>
     <row r="37" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F37" s="9" t="s">
@@ -2226,7 +2563,7 @@
       </c>
       <c r="G37" s="9"/>
       <c r="H37" s="12" t="n">
-        <f aca="false">G13</f>
+        <f aca="false">H30*H36</f>
         <v>0</v>
       </c>
       <c r="I37" s="12"/>
@@ -2236,8 +2573,11 @@
         <v>38</v>
       </c>
       <c r="G38" s="9"/>
-      <c r="H38" s="13"/>
-      <c r="I38" s="13"/>
+      <c r="H38" s="12" t="n">
+        <f aca="false">H30+H32+H33+H34+H35+H37</f>
+        <v>0</v>
+      </c>
+      <c r="I38" s="12"/>
     </row>
     <row r="39" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F39" s="9" t="s">
@@ -2245,65 +2585,71 @@
       </c>
       <c r="G39" s="9"/>
       <c r="H39" s="12" t="n">
-        <f aca="false">H36+H37-H38</f>
+        <f aca="false">G13</f>
         <v>0</v>
       </c>
       <c r="I39" s="12"/>
     </row>
-    <row r="41" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="9" t="s">
+    <row r="40" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F40" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="B41" s="9"/>
-      <c r="C41" s="4"/>
-      <c r="D41" s="4"/>
-      <c r="E41" s="14" t="s">
+      <c r="G40" s="9"/>
+      <c r="H40" s="13"/>
+      <c r="I40" s="13"/>
+    </row>
+    <row r="41" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F41" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="F41" s="14"/>
-      <c r="G41" s="14"/>
-      <c r="H41" s="4"/>
-      <c r="I41" s="4"/>
-    </row>
-    <row r="43" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="15" t="s">
+      <c r="G41" s="9"/>
+      <c r="H41" s="12" t="n">
+        <f aca="false">H38+H39-H40</f>
+        <v>0</v>
+      </c>
+      <c r="I41" s="12"/>
+    </row>
+    <row r="43" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="B43" s="15"/>
-      <c r="C43" s="15"/>
-      <c r="D43" s="15"/>
-      <c r="E43" s="15"/>
+      <c r="B43" s="9"/>
+      <c r="C43" s="4"/>
+      <c r="D43" s="4"/>
+      <c r="E43" s="15" t="s">
+        <v>43</v>
+      </c>
       <c r="F43" s="15"/>
       <c r="G43" s="15"/>
-      <c r="H43" s="15"/>
-      <c r="I43" s="15"/>
-    </row>
-    <row r="44" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="15"/>
-      <c r="B44" s="15"/>
-      <c r="C44" s="15"/>
-      <c r="D44" s="15"/>
-      <c r="E44" s="15"/>
-      <c r="F44" s="15"/>
-      <c r="G44" s="15"/>
-      <c r="H44" s="15"/>
-      <c r="I44" s="15"/>
+      <c r="H43" s="4"/>
+      <c r="I43" s="4"/>
     </row>
     <row r="45" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="15"/>
-      <c r="B45" s="15"/>
-      <c r="C45" s="15"/>
-      <c r="D45" s="15"/>
-      <c r="E45" s="15"/>
-      <c r="F45" s="15"/>
-      <c r="G45" s="15"/>
-      <c r="H45" s="15"/>
-      <c r="I45" s="15"/>
-    </row>
-    <row r="47" customFormat="false" ht="11.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="16" t="s">
-        <v>43</v>
-      </c>
+      <c r="A45" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="B45" s="16"/>
+      <c r="C45" s="16"/>
+      <c r="D45" s="16"/>
+      <c r="E45" s="16"/>
+      <c r="F45" s="16"/>
+      <c r="G45" s="16"/>
+      <c r="H45" s="16"/>
+      <c r="I45" s="16"/>
+    </row>
+    <row r="46" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="16"/>
+      <c r="B46" s="16"/>
+      <c r="C46" s="16"/>
+      <c r="D46" s="16"/>
+      <c r="E46" s="16"/>
+      <c r="F46" s="16"/>
+      <c r="G46" s="16"/>
+      <c r="H46" s="16"/>
+      <c r="I46" s="16"/>
+    </row>
+    <row r="47" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="16"/>
       <c r="B47" s="16"/>
       <c r="C47" s="16"/>
       <c r="D47" s="16"/>
@@ -2313,8 +2659,21 @@
       <c r="H47" s="16"/>
       <c r="I47" s="16"/>
     </row>
+    <row r="49" customFormat="false" ht="11.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="B49" s="17"/>
+      <c r="C49" s="17"/>
+      <c r="D49" s="17"/>
+      <c r="E49" s="17"/>
+      <c r="F49" s="17"/>
+      <c r="G49" s="17"/>
+      <c r="H49" s="17"/>
+      <c r="I49" s="17"/>
+    </row>
   </sheetData>
-  <mergeCells count="66">
+  <mergeCells count="70">
     <mergeCell ref="A1:D5"/>
     <mergeCell ref="G1:I1"/>
     <mergeCell ref="G2:I2"/>
@@ -2375,12 +2734,16 @@
     <mergeCell ref="H38:I38"/>
     <mergeCell ref="F39:G39"/>
     <mergeCell ref="H39:I39"/>
-    <mergeCell ref="A41:B41"/>
-    <mergeCell ref="C41:D41"/>
-    <mergeCell ref="E41:G41"/>
+    <mergeCell ref="F40:G40"/>
+    <mergeCell ref="H40:I40"/>
+    <mergeCell ref="F41:G41"/>
     <mergeCell ref="H41:I41"/>
-    <mergeCell ref="A43:I45"/>
-    <mergeCell ref="A47:I47"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="E43:G43"/>
+    <mergeCell ref="H43:I43"/>
+    <mergeCell ref="A45:I47"/>
+    <mergeCell ref="A49:I49"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.4" right="0.4" top="0.4" bottom="0.4" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2399,7 +2762,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B37"/>
+  <dimension ref="A1:B41"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -2407,219 +2770,247 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="B1" s="18"/>
+      <c r="A1" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" s="19"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="s">
-        <v>45</v>
-      </c>
-      <c r="B3" s="20" t="s">
-        <v>46</v>
+      <c r="A3" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="B3" s="21" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="21" t="s">
-        <v>47</v>
-      </c>
-      <c r="B5" s="22"/>
+      <c r="A5" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="B5" s="23"/>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="20" t="s">
-        <v>48</v>
-      </c>
-      <c r="B6" s="20" t="s">
-        <v>49</v>
+      <c r="A6" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="B6" s="21" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="20"/>
-      <c r="B7" s="23" t="s">
-        <v>50</v>
+      <c r="A7" s="21"/>
+      <c r="B7" s="24" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="20"/>
-      <c r="B8" s="23" t="s">
-        <v>51</v>
+      <c r="A8" s="21"/>
+      <c r="B8" s="24" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="21" t="s">
-        <v>52</v>
-      </c>
-      <c r="B10" s="22"/>
+      <c r="A10" s="22" t="s">
+        <v>54</v>
+      </c>
+      <c r="B10" s="23"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="20" t="s">
-        <v>53</v>
-      </c>
-      <c r="B11" s="20" t="s">
-        <v>54</v>
+      <c r="A11" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="B11" s="21" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="20" t="s">
-        <v>55</v>
-      </c>
-      <c r="B12" s="20" t="s">
-        <v>56</v>
+      <c r="A12" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="B12" s="21" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="B14" s="22"/>
+      <c r="A14" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="B14" s="23"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="B15" s="23" t="s">
-        <v>59</v>
+      <c r="A15" s="25" t="s">
+        <v>60</v>
+      </c>
+      <c r="B15" s="24" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="25"/>
-      <c r="B16" s="26" t="s">
-        <v>60</v>
+      <c r="A16" s="26"/>
+      <c r="B16" s="27" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="24" t="s">
-        <v>61</v>
-      </c>
-      <c r="B17" s="23" t="s">
-        <v>62</v>
+      <c r="A17" s="25" t="s">
+        <v>63</v>
+      </c>
+      <c r="B17" s="24" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="25"/>
-      <c r="B18" s="26" t="s">
-        <v>63</v>
+      <c r="A18" s="26"/>
+      <c r="B18" s="27" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="24" t="s">
+      <c r="A19" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="23" t="s">
-        <v>64</v>
+      <c r="B19" s="24" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="25"/>
-      <c r="B20" s="26" t="s">
-        <v>65</v>
+      <c r="A20" s="26"/>
+      <c r="B20" s="27" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="24" t="s">
-        <v>66</v>
-      </c>
-      <c r="B21" s="23" t="s">
-        <v>67</v>
+      <c r="A21" s="25" t="s">
+        <v>68</v>
+      </c>
+      <c r="B21" s="24" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="25"/>
-      <c r="B22" s="26" t="s">
+      <c r="A22" s="26"/>
+      <c r="B22" s="27" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="25" t="s">
+        <v>71</v>
+      </c>
+      <c r="B23" s="24" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="26"/>
+      <c r="B24" s="27" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="B25" s="24" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="26"/>
+      <c r="B26" s="27" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="25" t="s">
+        <v>77</v>
+      </c>
+      <c r="B27" s="24" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="26"/>
+      <c r="B28" s="27" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="25" t="s">
+        <v>20</v>
+      </c>
+      <c r="B29" s="24" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="26"/>
+      <c r="B30" s="27" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="22" t="s">
+        <v>82</v>
+      </c>
+      <c r="B32" s="23"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="B33" s="24" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="21" t="s">
+        <v>85</v>
+      </c>
+      <c r="B34" s="24" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="21"/>
+      <c r="B35" s="24" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="B36" s="24" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="24" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="24" t="s">
-        <v>69</v>
-      </c>
-      <c r="B23" s="23" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="25"/>
-      <c r="B24" s="26" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="24" t="s">
-        <v>72</v>
-      </c>
-      <c r="B25" s="23" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="25"/>
-      <c r="B26" s="26" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="B27" s="23" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="25"/>
-      <c r="B28" s="26" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="21" t="s">
-        <v>77</v>
-      </c>
-      <c r="B30" s="22"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="20" t="s">
-        <v>78</v>
-      </c>
-      <c r="B31" s="23" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="20" t="s">
-        <v>80</v>
-      </c>
-      <c r="B32" s="23" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="20"/>
-      <c r="B33" s="23" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="20" t="s">
-        <v>83</v>
-      </c>
-      <c r="B34" s="23" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="20"/>
-      <c r="B35" s="20" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="19" t="s">
-        <v>86</v>
-      </c>
-      <c r="B37" s="23" t="s">
-        <v>87</v>
+      <c r="B37" s="21" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="21"/>
+      <c r="B38" s="24" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="21"/>
+      <c r="B39" s="21" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="20" t="s">
+        <v>93</v>
+      </c>
+      <c r="B41" s="24" t="s">
+        <v>94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add dealership details to the empty lower-left area
Three centered lines above the approval row, bottom-aligned with the
money column: company name, street address, and phone/fax.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0163XvMSENuP7J3Nt4ti5Htq
</commit_message>
<xml_diff>
--- a/Buyers_Order_Worksheet_Template.xlsx
+++ b/Buyers_Order_Worksheet_Template.xlsx
@@ -298,7 +298,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="98">
   <si>
     <t xml:space="preserve">Date:</t>
   </si>
@@ -417,10 +417,19 @@
     <t xml:space="preserve">Total Price:</t>
   </si>
   <si>
+    <t xml:space="preserve">EXCELLENT AUTO SALES AND LEASING</t>
+  </si>
+  <si>
     <t xml:space="preserve">Trade Payoff:</t>
   </si>
   <si>
+    <t xml:space="preserve">6419 ALONDRA BLVD PARAMOUNT CA 90723</t>
+  </si>
+  <si>
     <t xml:space="preserve">Deposit:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tel: (310)906-8117    Fax: (562)529-7997</t>
   </si>
   <si>
     <t xml:space="preserve">Balance:</t>
@@ -1525,7 +1534,7 @@
     <numFmt numFmtId="168" formatCode="&quot;($&quot;#,##0.00\);&quot;($&quot;#,##0.00\);&quot;($0.00)&quot;"/>
     <numFmt numFmtId="169" formatCode="0.000%"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1573,6 +1582,21 @@
     </font>
     <font>
       <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="9.5"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="0"/>
@@ -1687,7 +1711,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -1723,6 +1747,13 @@
       <bottom style="medium"/>
       <diagonal/>
     </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -1749,7 +1780,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1810,27 +1841,27 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1838,7 +1869,15 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1846,7 +1885,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1854,11 +1893,11 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2580,8 +2619,14 @@
       <c r="I38" s="12"/>
     </row>
     <row r="39" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="B39" s="15"/>
+      <c r="C39" s="15"/>
+      <c r="D39" s="15"/>
       <c r="F39" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G39" s="9"/>
       <c r="H39" s="12" t="n">
@@ -2590,17 +2635,29 @@
       </c>
       <c r="I39" s="12"/>
     </row>
-    <row r="40" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="B40" s="16"/>
+      <c r="C40" s="16"/>
+      <c r="D40" s="16"/>
       <c r="F40" s="9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G40" s="9"/>
       <c r="H40" s="13"/>
       <c r="I40" s="13"/>
     </row>
-    <row r="41" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="B41" s="16"/>
+      <c r="C41" s="16"/>
+      <c r="D41" s="16"/>
       <c r="F41" s="9" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="G41" s="9"/>
       <c r="H41" s="12" t="n">
@@ -2611,69 +2668,69 @@
     </row>
     <row r="43" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="9" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B43" s="9"/>
       <c r="C43" s="4"/>
       <c r="D43" s="4"/>
-      <c r="E43" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="F43" s="15"/>
-      <c r="G43" s="15"/>
+      <c r="E43" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="F43" s="17"/>
+      <c r="G43" s="17"/>
       <c r="H43" s="4"/>
       <c r="I43" s="4"/>
     </row>
     <row r="45" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="B45" s="16"/>
-      <c r="C45" s="16"/>
-      <c r="D45" s="16"/>
-      <c r="E45" s="16"/>
-      <c r="F45" s="16"/>
-      <c r="G45" s="16"/>
-      <c r="H45" s="16"/>
-      <c r="I45" s="16"/>
+      <c r="A45" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="B45" s="18"/>
+      <c r="C45" s="18"/>
+      <c r="D45" s="18"/>
+      <c r="E45" s="18"/>
+      <c r="F45" s="18"/>
+      <c r="G45" s="18"/>
+      <c r="H45" s="18"/>
+      <c r="I45" s="18"/>
     </row>
     <row r="46" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="16"/>
-      <c r="B46" s="16"/>
-      <c r="C46" s="16"/>
-      <c r="D46" s="16"/>
-      <c r="E46" s="16"/>
-      <c r="F46" s="16"/>
-      <c r="G46" s="16"/>
-      <c r="H46" s="16"/>
-      <c r="I46" s="16"/>
+      <c r="A46" s="18"/>
+      <c r="B46" s="18"/>
+      <c r="C46" s="18"/>
+      <c r="D46" s="18"/>
+      <c r="E46" s="18"/>
+      <c r="F46" s="18"/>
+      <c r="G46" s="18"/>
+      <c r="H46" s="18"/>
+      <c r="I46" s="18"/>
     </row>
     <row r="47" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="16"/>
-      <c r="B47" s="16"/>
-      <c r="C47" s="16"/>
-      <c r="D47" s="16"/>
-      <c r="E47" s="16"/>
-      <c r="F47" s="16"/>
-      <c r="G47" s="16"/>
-      <c r="H47" s="16"/>
-      <c r="I47" s="16"/>
+      <c r="A47" s="18"/>
+      <c r="B47" s="18"/>
+      <c r="C47" s="18"/>
+      <c r="D47" s="18"/>
+      <c r="E47" s="18"/>
+      <c r="F47" s="18"/>
+      <c r="G47" s="18"/>
+      <c r="H47" s="18"/>
+      <c r="I47" s="18"/>
     </row>
     <row r="49" customFormat="false" ht="11.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="17" t="s">
-        <v>45</v>
-      </c>
-      <c r="B49" s="17"/>
-      <c r="C49" s="17"/>
-      <c r="D49" s="17"/>
-      <c r="E49" s="17"/>
-      <c r="F49" s="17"/>
-      <c r="G49" s="17"/>
-      <c r="H49" s="17"/>
-      <c r="I49" s="17"/>
+      <c r="A49" s="19" t="s">
+        <v>48</v>
+      </c>
+      <c r="B49" s="19"/>
+      <c r="C49" s="19"/>
+      <c r="D49" s="19"/>
+      <c r="E49" s="19"/>
+      <c r="F49" s="19"/>
+      <c r="G49" s="19"/>
+      <c r="H49" s="19"/>
+      <c r="I49" s="19"/>
     </row>
   </sheetData>
-  <mergeCells count="70">
+  <mergeCells count="73">
     <mergeCell ref="A1:D5"/>
     <mergeCell ref="G1:I1"/>
     <mergeCell ref="G2:I2"/>
@@ -2732,10 +2789,13 @@
     <mergeCell ref="H37:I37"/>
     <mergeCell ref="F38:G38"/>
     <mergeCell ref="H38:I38"/>
+    <mergeCell ref="A39:D39"/>
     <mergeCell ref="F39:G39"/>
     <mergeCell ref="H39:I39"/>
+    <mergeCell ref="A40:D40"/>
     <mergeCell ref="F40:G40"/>
     <mergeCell ref="H40:I40"/>
+    <mergeCell ref="A41:D41"/>
     <mergeCell ref="F41:G41"/>
     <mergeCell ref="H41:I41"/>
     <mergeCell ref="A43:B43"/>
@@ -2770,247 +2830,247 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="18" t="s">
-        <v>46</v>
-      </c>
-      <c r="B1" s="19"/>
+      <c r="A1" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" s="21"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="20" t="s">
-        <v>47</v>
-      </c>
-      <c r="B3" s="21" t="s">
-        <v>48</v>
+      <c r="A3" s="22" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3" s="23" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="22" t="s">
-        <v>49</v>
-      </c>
-      <c r="B5" s="23"/>
+      <c r="A5" s="24" t="s">
+        <v>52</v>
+      </c>
+      <c r="B5" s="25"/>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="21" t="s">
-        <v>50</v>
-      </c>
-      <c r="B6" s="21" t="s">
-        <v>51</v>
+      <c r="A6" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="B6" s="23" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="21"/>
-      <c r="B7" s="24" t="s">
-        <v>52</v>
+      <c r="A7" s="23"/>
+      <c r="B7" s="26" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="21"/>
-      <c r="B8" s="24" t="s">
-        <v>53</v>
+      <c r="A8" s="23"/>
+      <c r="B8" s="26" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="22" t="s">
-        <v>54</v>
-      </c>
-      <c r="B10" s="23"/>
+      <c r="A10" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="B10" s="25"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="21" t="s">
-        <v>55</v>
-      </c>
-      <c r="B11" s="21" t="s">
-        <v>56</v>
+      <c r="A11" s="23" t="s">
+        <v>58</v>
+      </c>
+      <c r="B11" s="23" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="B12" s="21" t="s">
-        <v>58</v>
+      <c r="A12" s="23" t="s">
+        <v>60</v>
+      </c>
+      <c r="B12" s="23" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="22" t="s">
-        <v>59</v>
-      </c>
-      <c r="B14" s="23"/>
+      <c r="A14" s="24" t="s">
+        <v>62</v>
+      </c>
+      <c r="B14" s="25"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="25" t="s">
-        <v>60</v>
-      </c>
-      <c r="B15" s="24" t="s">
-        <v>61</v>
+      <c r="A15" s="27" t="s">
+        <v>63</v>
+      </c>
+      <c r="B15" s="26" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="26"/>
-      <c r="B16" s="27" t="s">
-        <v>62</v>
+      <c r="A16" s="28"/>
+      <c r="B16" s="29" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="25" t="s">
-        <v>63</v>
-      </c>
-      <c r="B17" s="24" t="s">
-        <v>64</v>
+      <c r="A17" s="27" t="s">
+        <v>66</v>
+      </c>
+      <c r="B17" s="26" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="26"/>
-      <c r="B18" s="27" t="s">
-        <v>65</v>
+      <c r="A18" s="28"/>
+      <c r="B18" s="29" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="25" t="s">
+      <c r="A19" s="27" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="24" t="s">
-        <v>66</v>
+      <c r="B19" s="26" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="26"/>
-      <c r="B20" s="27" t="s">
-        <v>67</v>
+      <c r="A20" s="28"/>
+      <c r="B20" s="29" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="25" t="s">
-        <v>68</v>
-      </c>
-      <c r="B21" s="24" t="s">
-        <v>69</v>
+      <c r="A21" s="27" t="s">
+        <v>71</v>
+      </c>
+      <c r="B21" s="26" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="26"/>
-      <c r="B22" s="27" t="s">
-        <v>70</v>
+      <c r="A22" s="28"/>
+      <c r="B22" s="29" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="25" t="s">
+      <c r="A23" s="27" t="s">
+        <v>74</v>
+      </c>
+      <c r="B23" s="26" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="28"/>
+      <c r="B24" s="29" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="27" t="s">
+        <v>77</v>
+      </c>
+      <c r="B25" s="26" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="28"/>
+      <c r="B26" s="29" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="27" t="s">
+        <v>80</v>
+      </c>
+      <c r="B27" s="26" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="28"/>
+      <c r="B28" s="29" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B29" s="26" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="28"/>
+      <c r="B30" s="29" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="24" t="s">
+        <v>85</v>
+      </c>
+      <c r="B32" s="25"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="B33" s="26" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="23" t="s">
+        <v>88</v>
+      </c>
+      <c r="B34" s="26" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="23"/>
+      <c r="B35" s="26" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="23" t="s">
+        <v>91</v>
+      </c>
+      <c r="B36" s="26" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="26" t="s">
         <v>71</v>
       </c>
-      <c r="B23" s="24" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="26"/>
-      <c r="B24" s="27" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="25" t="s">
-        <v>74</v>
-      </c>
-      <c r="B25" s="24" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="26"/>
-      <c r="B26" s="27" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="25" t="s">
-        <v>77</v>
-      </c>
-      <c r="B27" s="24" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="26"/>
-      <c r="B28" s="27" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="B29" s="24" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="26"/>
-      <c r="B30" s="27" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="22" t="s">
-        <v>82</v>
-      </c>
-      <c r="B32" s="23"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="21" t="s">
-        <v>83</v>
-      </c>
-      <c r="B33" s="24" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="21" t="s">
-        <v>85</v>
-      </c>
-      <c r="B34" s="24" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="21"/>
-      <c r="B35" s="24" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="21" t="s">
-        <v>88</v>
-      </c>
-      <c r="B36" s="24" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="24" t="s">
-        <v>68</v>
-      </c>
-      <c r="B37" s="21" t="s">
-        <v>90</v>
+      <c r="B37" s="23" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="21"/>
-      <c r="B38" s="24" t="s">
-        <v>91</v>
+      <c r="A38" s="23"/>
+      <c r="B38" s="26" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="21"/>
-      <c r="B39" s="21" t="s">
-        <v>92</v>
+      <c r="A39" s="23"/>
+      <c r="B39" s="23" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="20" t="s">
-        <v>93</v>
-      </c>
-      <c r="B41" s="24" t="s">
-        <v>94</v>
+      <c r="A41" s="22" t="s">
+        <v>96</v>
+      </c>
+      <c r="B41" s="26" t="s">
+        <v>97</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove the customer and management approval row
Both signature labels and their input fields are dropped; the disclaimer
now follows directly after the totals and the company block.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0163XvMSENuP7J3Nt4ti5Htq
</commit_message>
<xml_diff>
--- a/Buyers_Order_Worksheet_Template.xlsx
+++ b/Buyers_Order_Worksheet_Template.xlsx
@@ -12,7 +12,7 @@
     <sheet name="README (使い方・計算式)" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">'Buyers Order'!$A$1:$I$49</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">'Buyers Order'!$A$1:$I$47</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -298,7 +298,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="96">
   <si>
     <t xml:space="preserve">Date:</t>
   </si>
@@ -433,12 +433,6 @@
   </si>
   <si>
     <t xml:space="preserve">Balance:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Customer Approval:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Management Approval:</t>
   </si>
   <si>
     <t xml:space="preserve">By signing this authorization form, you certify that the above personal information is correct and accurate, and authorize the release of credit and employment information. By signing above, I provide to the dealership and its affiliates consent to communicate with me about my vehicle or any future vehicles using electronic verbal and written communications including but not limited to email, text messaging, SMS, phone calls and direct mail. Terms and conditions subject to credit approval. For information only. This is not an offer or contract for sale.</t>
@@ -1780,7 +1774,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="29">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1847,10 +1841,6 @@
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -2232,7 +2222,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
@@ -2666,47 +2656,45 @@
       </c>
       <c r="I41" s="12"/>
     </row>
-    <row r="43" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="9" t="s">
+    <row r="43" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="B43" s="9"/>
-      <c r="C43" s="4"/>
-      <c r="D43" s="4"/>
-      <c r="E43" s="17" t="s">
-        <v>46</v>
-      </c>
+      <c r="B43" s="17"/>
+      <c r="C43" s="17"/>
+      <c r="D43" s="17"/>
+      <c r="E43" s="17"/>
       <c r="F43" s="17"/>
       <c r="G43" s="17"/>
-      <c r="H43" s="4"/>
-      <c r="I43" s="4"/>
+      <c r="H43" s="17"/>
+      <c r="I43" s="17"/>
+    </row>
+    <row r="44" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="17"/>
+      <c r="B44" s="17"/>
+      <c r="C44" s="17"/>
+      <c r="D44" s="17"/>
+      <c r="E44" s="17"/>
+      <c r="F44" s="17"/>
+      <c r="G44" s="17"/>
+      <c r="H44" s="17"/>
+      <c r="I44" s="17"/>
     </row>
     <row r="45" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="18" t="s">
-        <v>47</v>
-      </c>
-      <c r="B45" s="18"/>
-      <c r="C45" s="18"/>
-      <c r="D45" s="18"/>
-      <c r="E45" s="18"/>
-      <c r="F45" s="18"/>
-      <c r="G45" s="18"/>
-      <c r="H45" s="18"/>
-      <c r="I45" s="18"/>
-    </row>
-    <row r="46" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="18"/>
-      <c r="B46" s="18"/>
-      <c r="C46" s="18"/>
-      <c r="D46" s="18"/>
-      <c r="E46" s="18"/>
-      <c r="F46" s="18"/>
-      <c r="G46" s="18"/>
-      <c r="H46" s="18"/>
-      <c r="I46" s="18"/>
-    </row>
-    <row r="47" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="18"/>
+      <c r="A45" s="17"/>
+      <c r="B45" s="17"/>
+      <c r="C45" s="17"/>
+      <c r="D45" s="17"/>
+      <c r="E45" s="17"/>
+      <c r="F45" s="17"/>
+      <c r="G45" s="17"/>
+      <c r="H45" s="17"/>
+      <c r="I45" s="17"/>
+    </row>
+    <row r="47" customFormat="false" ht="11.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="18" t="s">
+        <v>46</v>
+      </c>
       <c r="B47" s="18"/>
       <c r="C47" s="18"/>
       <c r="D47" s="18"/>
@@ -2716,21 +2704,8 @@
       <c r="H47" s="18"/>
       <c r="I47" s="18"/>
     </row>
-    <row r="49" customFormat="false" ht="11.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="19" t="s">
-        <v>48</v>
-      </c>
-      <c r="B49" s="19"/>
-      <c r="C49" s="19"/>
-      <c r="D49" s="19"/>
-      <c r="E49" s="19"/>
-      <c r="F49" s="19"/>
-      <c r="G49" s="19"/>
-      <c r="H49" s="19"/>
-      <c r="I49" s="19"/>
-    </row>
   </sheetData>
-  <mergeCells count="73">
+  <mergeCells count="69">
     <mergeCell ref="A1:D5"/>
     <mergeCell ref="G1:I1"/>
     <mergeCell ref="G2:I2"/>
@@ -2798,12 +2773,8 @@
     <mergeCell ref="A41:D41"/>
     <mergeCell ref="F41:G41"/>
     <mergeCell ref="H41:I41"/>
-    <mergeCell ref="A43:B43"/>
-    <mergeCell ref="C43:D43"/>
-    <mergeCell ref="E43:G43"/>
-    <mergeCell ref="H43:I43"/>
-    <mergeCell ref="A45:I47"/>
-    <mergeCell ref="A49:I49"/>
+    <mergeCell ref="A43:I45"/>
+    <mergeCell ref="A47:I47"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="true"/>
   <pageMargins left="0.4" right="0.4" top="0.4" bottom="0.4" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2830,247 +2801,247 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" s="20"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="B3" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="21"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="22" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="23" t="s">
         <v>50</v>
       </c>
-      <c r="B3" s="23" t="s">
+      <c r="B5" s="24"/>
+    </row>
+    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="22" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="24" t="s">
+      <c r="B6" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="B5" s="25"/>
-    </row>
-    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="23" t="s">
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="22"/>
+      <c r="B7" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="B6" s="23" t="s">
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="22"/>
+      <c r="B8" s="25" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="23"/>
-      <c r="B7" s="26" t="s">
+    <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="23" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="23"/>
-      <c r="B8" s="26" t="s">
+      <c r="B10" s="24"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="22" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="24" t="s">
+      <c r="B11" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="B10" s="25"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="23" t="s">
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="B11" s="23" t="s">
+      <c r="B12" s="22" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="23" t="s">
+    <row r="14" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="23" t="s">
         <v>60</v>
       </c>
-      <c r="B12" s="23" t="s">
+      <c r="B14" s="24"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="26" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="24" t="s">
+      <c r="B15" s="25" t="s">
         <v>62</v>
       </c>
-      <c r="B14" s="25"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="27" t="s">
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="27"/>
+      <c r="B16" s="28" t="s">
         <v>63</v>
       </c>
-      <c r="B15" s="26" t="s">
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="26" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="28"/>
-      <c r="B16" s="29" t="s">
+      <c r="B17" s="25" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="27" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="27"/>
+      <c r="B18" s="28" t="s">
         <v>66</v>
       </c>
-      <c r="B17" s="26" t="s">
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="26" t="s">
+        <v>31</v>
+      </c>
+      <c r="B19" s="25" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="28"/>
-      <c r="B18" s="29" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="27"/>
+      <c r="B20" s="28" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="27" t="s">
-        <v>31</v>
-      </c>
-      <c r="B19" s="26" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="26" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="28"/>
-      <c r="B20" s="29" t="s">
+      <c r="B21" s="25" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="27" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="27"/>
+      <c r="B22" s="28" t="s">
         <v>71</v>
       </c>
-      <c r="B21" s="26" t="s">
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="26" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="28"/>
-      <c r="B22" s="29" t="s">
+      <c r="B23" s="25" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="27" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="27"/>
+      <c r="B24" s="28" t="s">
         <v>74</v>
       </c>
-      <c r="B23" s="26" t="s">
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="26" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="28"/>
-      <c r="B24" s="29" t="s">
+      <c r="B25" s="25" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="27" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="27"/>
+      <c r="B26" s="28" t="s">
         <v>77</v>
       </c>
-      <c r="B25" s="26" t="s">
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="26" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="28"/>
-      <c r="B26" s="29" t="s">
+      <c r="B27" s="25" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="27" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="27"/>
+      <c r="B28" s="28" t="s">
         <v>80</v>
       </c>
-      <c r="B27" s="26" t="s">
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="B29" s="25" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="28"/>
-      <c r="B28" s="29" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="27"/>
+      <c r="B30" s="28" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="27" t="s">
-        <v>20</v>
-      </c>
-      <c r="B29" s="26" t="s">
+    <row r="32" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="23" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="28"/>
-      <c r="B30" s="29" t="s">
+      <c r="B32" s="24"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="22" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="32" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="24" t="s">
+      <c r="B33" s="25" t="s">
         <v>85</v>
       </c>
-      <c r="B32" s="25"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="23" t="s">
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="B33" s="26" t="s">
+      <c r="B34" s="25" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="23" t="s">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="22"/>
+      <c r="B35" s="25" t="s">
         <v>88</v>
       </c>
-      <c r="B34" s="26" t="s">
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="22" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="23"/>
-      <c r="B35" s="26" t="s">
+      <c r="B36" s="25" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="23" t="s">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="25" t="s">
+        <v>69</v>
+      </c>
+      <c r="B37" s="22" t="s">
         <v>91</v>
       </c>
-      <c r="B36" s="26" t="s">
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="22"/>
+      <c r="B38" s="25" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="26" t="s">
-        <v>71</v>
-      </c>
-      <c r="B37" s="23" t="s">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="22"/>
+      <c r="B39" s="22" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="23"/>
-      <c r="B38" s="26" t="s">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="21" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="23"/>
-      <c r="B39" s="23" t="s">
+      <c r="B41" s="25" t="s">
         <v>95</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="22" t="s">
-        <v>96</v>
-      </c>
-      <c r="B41" s="26" t="s">
-        <v>97</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Restore the approval row and drop the yellow input shading
- Customer Approval and Management Approval fields are back
- Input cells are white instead of yellow; blue text on the underline
  still marks them as fill-in fields
- Legend and README updated to describe the color coding by font color

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0163XvMSENuP7J3Nt4ti5Htq
</commit_message>
<xml_diff>
--- a/Buyers_Order_Worksheet_Template.xlsx
+++ b/Buyers_Order_Worksheet_Template.xlsx
@@ -12,7 +12,7 @@
     <sheet name="README (使い方・計算式)" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">'Buyers Order'!$A$1:$I$47</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">'Buyers Order'!$A$1:$I$49</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -298,7 +298,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="98">
   <si>
     <t xml:space="preserve">Date:</t>
   </si>
@@ -433,6 +433,12 @@
   </si>
   <si>
     <t xml:space="preserve">Balance:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customer Approval:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Management Approval:</t>
   </si>
   <si>
     <t xml:space="preserve">By signing this authorization form, you certify that the above personal information is correct and accurate, and authorize the release of credit and employment information. By signing above, I provide to the dealership and its affiliates consent to communicate with me about my vehicle or any future vehicles using electronic verbal and written communications including but not limited to email, text messaging, SMS, phone calls and direct mail. Terms and conditions subject to credit approval. For information only. This is not an offer or contract for sale.</t>
@@ -467,7 +473,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">黄色＋青文字 </t>
+      <t xml:space="preserve">青文字 </t>
     </r>
     <r>
       <rPr>
@@ -509,7 +515,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">黒文字・塗りなし </t>
+      <t xml:space="preserve">黒文字 </t>
     </r>
     <r>
       <rPr>
@@ -827,67 +833,13 @@
     <t xml:space="preserve">■ セルの色分け</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">黄色 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">+ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">青文字</t>
-    </r>
+    <t xml:space="preserve">青文字</t>
   </si>
   <si>
     <t xml:space="preserve">手入力セル。ここだけを入力してください。</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">白 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">+ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">黒文字</t>
-    </r>
+    <t xml:space="preserve">黒文字</t>
   </si>
   <si>
     <t xml:space="preserve">計算式セル。自動計算されるので編集しないでください。</t>
@@ -1304,7 +1256,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">（黄色）に州・郡市の合計税率を入力すると自動計算され、</t>
+      <t xml:space="preserve">（青文字の記入欄）に州・郡市の合計税率を入力すると自動計算され、</t>
     </r>
   </si>
   <si>
@@ -1700,7 +1652,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF99"/>
+        <fgColor rgb="FFFFFFFF"/>
         <bgColor rgb="FFFFFFCC"/>
       </patternFill>
     </fill>
@@ -1774,7 +1726,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1841,6 +1793,10 @@
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -2222,7 +2178,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
@@ -2656,45 +2612,47 @@
       </c>
       <c r="I41" s="12"/>
     </row>
-    <row r="43" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="17" t="s">
+    <row r="43" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="B43" s="17"/>
-      <c r="C43" s="17"/>
-      <c r="D43" s="17"/>
-      <c r="E43" s="17"/>
+      <c r="B43" s="9"/>
+      <c r="C43" s="4"/>
+      <c r="D43" s="4"/>
+      <c r="E43" s="17" t="s">
+        <v>46</v>
+      </c>
       <c r="F43" s="17"/>
       <c r="G43" s="17"/>
-      <c r="H43" s="17"/>
-      <c r="I43" s="17"/>
-    </row>
-    <row r="44" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="17"/>
-      <c r="B44" s="17"/>
-      <c r="C44" s="17"/>
-      <c r="D44" s="17"/>
-      <c r="E44" s="17"/>
-      <c r="F44" s="17"/>
-      <c r="G44" s="17"/>
-      <c r="H44" s="17"/>
-      <c r="I44" s="17"/>
+      <c r="H43" s="4"/>
+      <c r="I43" s="4"/>
     </row>
     <row r="45" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="17"/>
-      <c r="B45" s="17"/>
-      <c r="C45" s="17"/>
-      <c r="D45" s="17"/>
-      <c r="E45" s="17"/>
-      <c r="F45" s="17"/>
-      <c r="G45" s="17"/>
-      <c r="H45" s="17"/>
-      <c r="I45" s="17"/>
-    </row>
-    <row r="47" customFormat="false" ht="11.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="18" t="s">
-        <v>46</v>
-      </c>
+      <c r="A45" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="B45" s="18"/>
+      <c r="C45" s="18"/>
+      <c r="D45" s="18"/>
+      <c r="E45" s="18"/>
+      <c r="F45" s="18"/>
+      <c r="G45" s="18"/>
+      <c r="H45" s="18"/>
+      <c r="I45" s="18"/>
+    </row>
+    <row r="46" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="18"/>
+      <c r="B46" s="18"/>
+      <c r="C46" s="18"/>
+      <c r="D46" s="18"/>
+      <c r="E46" s="18"/>
+      <c r="F46" s="18"/>
+      <c r="G46" s="18"/>
+      <c r="H46" s="18"/>
+      <c r="I46" s="18"/>
+    </row>
+    <row r="47" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="18"/>
       <c r="B47" s="18"/>
       <c r="C47" s="18"/>
       <c r="D47" s="18"/>
@@ -2704,8 +2662,21 @@
       <c r="H47" s="18"/>
       <c r="I47" s="18"/>
     </row>
+    <row r="49" customFormat="false" ht="11.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="19" t="s">
+        <v>48</v>
+      </c>
+      <c r="B49" s="19"/>
+      <c r="C49" s="19"/>
+      <c r="D49" s="19"/>
+      <c r="E49" s="19"/>
+      <c r="F49" s="19"/>
+      <c r="G49" s="19"/>
+      <c r="H49" s="19"/>
+      <c r="I49" s="19"/>
+    </row>
   </sheetData>
-  <mergeCells count="69">
+  <mergeCells count="73">
     <mergeCell ref="A1:D5"/>
     <mergeCell ref="G1:I1"/>
     <mergeCell ref="G2:I2"/>
@@ -2773,8 +2744,12 @@
     <mergeCell ref="A41:D41"/>
     <mergeCell ref="F41:G41"/>
     <mergeCell ref="H41:I41"/>
-    <mergeCell ref="A43:I45"/>
-    <mergeCell ref="A47:I47"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="E43:G43"/>
+    <mergeCell ref="H43:I43"/>
+    <mergeCell ref="A45:I47"/>
+    <mergeCell ref="A49:I49"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="true"/>
   <pageMargins left="0.4" right="0.4" top="0.4" bottom="0.4" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2801,247 +2776,247 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="B1" s="20"/>
+      <c r="A1" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" s="21"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="21" t="s">
-        <v>48</v>
-      </c>
-      <c r="B3" s="22" t="s">
-        <v>49</v>
+      <c r="A3" s="22" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3" s="23" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="23" t="s">
-        <v>50</v>
-      </c>
-      <c r="B5" s="24"/>
+      <c r="A5" s="24" t="s">
+        <v>52</v>
+      </c>
+      <c r="B5" s="25"/>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="22" t="s">
-        <v>51</v>
-      </c>
-      <c r="B6" s="22" t="s">
-        <v>52</v>
+      <c r="A6" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="B6" s="23" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="22"/>
-      <c r="B7" s="25" t="s">
-        <v>53</v>
+      <c r="A7" s="23"/>
+      <c r="B7" s="26" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="22"/>
-      <c r="B8" s="25" t="s">
-        <v>54</v>
+      <c r="A8" s="23"/>
+      <c r="B8" s="26" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="23" t="s">
-        <v>55</v>
-      </c>
-      <c r="B10" s="24"/>
+      <c r="A10" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="B10" s="25"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="22" t="s">
-        <v>56</v>
-      </c>
-      <c r="B11" s="22" t="s">
-        <v>57</v>
+      <c r="A11" s="23" t="s">
+        <v>58</v>
+      </c>
+      <c r="B11" s="23" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="22" t="s">
-        <v>58</v>
-      </c>
-      <c r="B12" s="22" t="s">
-        <v>59</v>
+      <c r="A12" s="23" t="s">
+        <v>60</v>
+      </c>
+      <c r="B12" s="23" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="B14" s="24"/>
+      <c r="A14" s="24" t="s">
+        <v>62</v>
+      </c>
+      <c r="B14" s="25"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="26" t="s">
-        <v>61</v>
-      </c>
-      <c r="B15" s="25" t="s">
-        <v>62</v>
+      <c r="A15" s="27" t="s">
+        <v>63</v>
+      </c>
+      <c r="B15" s="26" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="27"/>
-      <c r="B16" s="28" t="s">
-        <v>63</v>
+      <c r="A16" s="28"/>
+      <c r="B16" s="29" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="26" t="s">
-        <v>64</v>
-      </c>
-      <c r="B17" s="25" t="s">
-        <v>65</v>
+      <c r="A17" s="27" t="s">
+        <v>66</v>
+      </c>
+      <c r="B17" s="26" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="27"/>
-      <c r="B18" s="28" t="s">
-        <v>66</v>
+      <c r="A18" s="28"/>
+      <c r="B18" s="29" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="26" t="s">
+      <c r="A19" s="27" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="25" t="s">
-        <v>67</v>
+      <c r="B19" s="26" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="27"/>
-      <c r="B20" s="28" t="s">
-        <v>68</v>
+      <c r="A20" s="28"/>
+      <c r="B20" s="29" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="26" t="s">
-        <v>69</v>
-      </c>
-      <c r="B21" s="25" t="s">
-        <v>70</v>
+      <c r="A21" s="27" t="s">
+        <v>71</v>
+      </c>
+      <c r="B21" s="26" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="27"/>
-      <c r="B22" s="28" t="s">
+      <c r="A22" s="28"/>
+      <c r="B22" s="29" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="27" t="s">
+        <v>74</v>
+      </c>
+      <c r="B23" s="26" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="28"/>
+      <c r="B24" s="29" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="27" t="s">
+        <v>77</v>
+      </c>
+      <c r="B25" s="26" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="28"/>
+      <c r="B26" s="29" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="27" t="s">
+        <v>80</v>
+      </c>
+      <c r="B27" s="26" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="28"/>
+      <c r="B28" s="29" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B29" s="26" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="28"/>
+      <c r="B30" s="29" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="24" t="s">
+        <v>85</v>
+      </c>
+      <c r="B32" s="25"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="B33" s="26" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="23" t="s">
+        <v>88</v>
+      </c>
+      <c r="B34" s="26" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="23"/>
+      <c r="B35" s="26" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="23" t="s">
+        <v>91</v>
+      </c>
+      <c r="B36" s="26" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="26" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="26" t="s">
-        <v>72</v>
-      </c>
-      <c r="B23" s="25" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="27"/>
-      <c r="B24" s="28" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="26" t="s">
-        <v>75</v>
-      </c>
-      <c r="B25" s="25" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="27"/>
-      <c r="B26" s="28" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="26" t="s">
-        <v>78</v>
-      </c>
-      <c r="B27" s="25" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="27"/>
-      <c r="B28" s="28" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B29" s="25" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="27"/>
-      <c r="B30" s="28" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="23" t="s">
-        <v>83</v>
-      </c>
-      <c r="B32" s="24"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="22" t="s">
-        <v>84</v>
-      </c>
-      <c r="B33" s="25" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="22" t="s">
-        <v>86</v>
-      </c>
-      <c r="B34" s="25" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="22"/>
-      <c r="B35" s="25" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="22" t="s">
-        <v>89</v>
-      </c>
-      <c r="B36" s="25" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="25" t="s">
-        <v>69</v>
-      </c>
-      <c r="B37" s="22" t="s">
-        <v>91</v>
+      <c r="B37" s="23" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="22"/>
-      <c r="B38" s="25" t="s">
-        <v>92</v>
+      <c r="A38" s="23"/>
+      <c r="B38" s="26" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="22"/>
-      <c r="B39" s="22" t="s">
-        <v>93</v>
+      <c r="A39" s="23"/>
+      <c r="B39" s="23" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="21" t="s">
-        <v>94</v>
-      </c>
-      <c r="B41" s="25" t="s">
-        <v>95</v>
+      <c r="A41" s="22" t="s">
+        <v>96</v>
+      </c>
+      <c r="B41" s="26" t="s">
+        <v>97</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Replace the drawn stand-in with the real Ford oval artwork
The badge is now rendered from the official mark's vector outline (the
ford.svg path shipped in the simple-icons npm package, CC0), cropped to
the oval with a small margin and rasterized at 1358x478. It is placed in
the LOGO 1 slot scaled to fit without distortion, and the hand-drawn
approximation is removed.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0163XvMSENuP7J3Nt4ti5Htq
</commit_message>
<xml_diff>
--- a/Buyers_Order_Worksheet_Template.xlsx
+++ b/Buyers_Order_Worksheet_Template.xlsx
@@ -1931,8 +1931,8 @@
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>272880</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>28080</xdr:rowOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>228240</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1946,7 +1946,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="1428480" cy="580680"/>
+          <a:ext cx="1428480" cy="504360"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>

<commit_message>
Keep the header logos inside their frame
Both pictures are now placed through one helper that fits them to a fixed
box while preserving aspect, and pins them with a single-cell anchor plus
an 8px inset from the cell corner instead of sitting flush against it.
The emblem shrinks to 125x44px so it stays well within the header block.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0163XvMSENuP7J3Nt4ti5Htq
</commit_message>
<xml_diff>
--- a/Buyers_Order_Worksheet_Template.xlsx
+++ b/Buyers_Order_Worksheet_Template.xlsx
@@ -1924,15 +1924,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>76320</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>76320</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>272880</xdr:colOff>
+      <xdr:colOff>110880</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>228240</xdr:rowOff>
+      <xdr:rowOff>218880</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1945,8 +1945,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="1428480" cy="504360"/>
+          <a:off x="76320" y="76320"/>
+          <a:ext cx="1190160" cy="418680"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1961,15 +1961,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>76320</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>76320</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>898200</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>28080</xdr:rowOff>
+      <xdr:colOff>450720</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>218880</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1982,8 +1982,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3467160" y="0"/>
-          <a:ext cx="1875960" cy="580680"/>
+          <a:off x="3543480" y="76320"/>
+          <a:ext cx="1352160" cy="418680"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>

<commit_message>
Keep the emblem inside column A
The picture was 125px wide against a 96px column, so its selection box
ran past column A into B. Shrink it to 84x30px with a 6px inset, which
leaves its right edge at 90px, and scale the second placeholder down to
the same header band.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0163XvMSENuP7J3Nt4ti5Htq
</commit_message>
<xml_diff>
--- a/Buyers_Order_Worksheet_Template.xlsx
+++ b/Buyers_Order_Worksheet_Template.xlsx
@@ -1924,15 +1924,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>76320</xdr:colOff>
+      <xdr:colOff>57240</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>76320</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>110880</xdr:colOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>857160</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>218880</xdr:rowOff>
+      <xdr:rowOff>85680</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1945,8 +1945,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="76320" y="76320"/>
-          <a:ext cx="1190160" cy="418680"/>
+          <a:off x="57240" y="76320"/>
+          <a:ext cx="799920" cy="285480"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1961,15 +1961,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>76320</xdr:colOff>
+      <xdr:colOff>57240</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>76320</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>450720</xdr:colOff>
+      <xdr:colOff>60120</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>218880</xdr:rowOff>
+      <xdr:rowOff>104760</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1982,8 +1982,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3543480" y="76320"/>
-          <a:ext cx="1352160" cy="418680"/>
+          <a:off x="3524400" y="76320"/>
+          <a:ext cx="980640" cy="304560"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>

<commit_message>
Stop the emblem from being clipped at its edges
The PNG was cropped to the oval's exact bounding box with only ~1% of
margin, so at 88px wide the outline had well under a pixel of clearance
and read as cut off. Re-render with 6% horizontal and 12% vertical
padding (1491x560) and refit it inside column A.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0163XvMSENuP7J3Nt4ti5Htq
</commit_message>
<xml_diff>
--- a/Buyers_Order_Worksheet_Template.xlsx
+++ b/Buyers_Order_Worksheet_Template.xlsx
@@ -1924,15 +1924,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>57240</xdr:colOff>
+      <xdr:colOff>38160</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>76320</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>857160</xdr:colOff>
+      <xdr:colOff>875880</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>85680</xdr:rowOff>
+      <xdr:rowOff>114120</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1945,8 +1945,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="57240" y="76320"/>
-          <a:ext cx="799920" cy="285480"/>
+          <a:off x="38160" y="76320"/>
+          <a:ext cx="837720" cy="313920"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>

<commit_message>
Print both forms on A4 with minimal margins, and use the color roundel
Page setup on both templates moves to A4 with 0.3in margins. Row heights
are scaled so the content's aspect matches the page, which fills the
sheet instead of leaving a third of it blank; the buyers order no longer
needs vertical centering. A measured correction factor converts openpyxl
width units to real inches, so the fit-to-page scale no longer shrinks
the layout away from the right margin.

The proposal's emblem is replaced with the color BMW roundel, rendered
from the bmw-logo.svg in the car-brand-logos npm package and cropped to
its alpha bounding box so it carries no padding of its own.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0163XvMSENuP7J3Nt4ti5Htq
</commit_message>
<xml_diff>
--- a/Buyers_Order_Worksheet_Template.xlsx
+++ b/Buyers_Order_Worksheet_Template.xlsx
@@ -1931,8 +1931,8 @@
     <xdr:to>
       <xdr:col>0</xdr:col>
       <xdr:colOff>875880</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>114120</xdr:rowOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>390240</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1968,8 +1968,8 @@
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>60120</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>104760</xdr:rowOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>380880</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2192,7 +2192,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="32.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2204,7 +2204,7 @@
       <c r="H1" s="3"/>
       <c r="I1" s="3"/>
     </row>
-    <row r="2" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="32.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -2216,7 +2216,7 @@
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
     </row>
-    <row r="3" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="32.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -2228,19 +2228,20 @@
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
     </row>
-    <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="32.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
     </row>
-    <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="32.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
     </row>
-    <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
         <v>3</v>
       </c>
@@ -2253,7 +2254,7 @@
       <c r="H7" s="5"/>
       <c r="I7" s="5"/>
     </row>
-    <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
         <v>4</v>
       </c>
@@ -2267,7 +2268,7 @@
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
     </row>
-    <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
         <v>6</v>
       </c>
@@ -2281,7 +2282,7 @@
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
     </row>
-    <row r="10" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -2295,7 +2296,8 @@
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
     </row>
-    <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
         <v>10</v>
       </c>
@@ -2309,7 +2311,7 @@
       <c r="H12" s="5"/>
       <c r="I12" s="5"/>
     </row>
-    <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
@@ -2325,7 +2327,7 @@
       <c r="H13" s="6"/>
       <c r="I13" s="6"/>
     </row>
-    <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
         <v>15</v>
       </c>
@@ -2339,7 +2341,7 @@
       <c r="H14" s="4"/>
       <c r="I14" s="4"/>
     </row>
-    <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
         <v>16</v>
       </c>
@@ -2353,7 +2355,7 @@
       <c r="H15" s="4"/>
       <c r="I15" s="4"/>
     </row>
-    <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
         <v>17</v>
       </c>
@@ -2367,7 +2369,7 @@
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
     </row>
-    <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
         <v>18</v>
       </c>
@@ -2385,7 +2387,8 @@
       </c>
       <c r="I17" s="4"/>
     </row>
-    <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="19" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
         <v>20</v>
       </c>
@@ -2399,7 +2402,7 @@
       <c r="H19" s="10"/>
       <c r="I19" s="10"/>
     </row>
-    <row r="20" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="n">
         <f aca="false">H41</f>
         <v>0</v>
@@ -2414,13 +2417,13 @@
       <c r="H20" s="10"/>
       <c r="I20" s="10"/>
     </row>
-    <row r="21" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="11"/>
       <c r="B21" s="11"/>
       <c r="C21" s="11"/>
       <c r="D21" s="11"/>
     </row>
-    <row r="22" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F22" s="9" t="s">
         <v>23</v>
       </c>
@@ -2431,7 +2434,7 @@
       </c>
       <c r="I22" s="12"/>
     </row>
-    <row r="23" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F23" s="9" t="s">
         <v>24</v>
       </c>
@@ -2439,7 +2442,7 @@
       <c r="H23" s="10"/>
       <c r="I23" s="10"/>
     </row>
-    <row r="24" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F24" s="9" t="s">
         <v>25</v>
       </c>
@@ -2447,7 +2450,7 @@
       <c r="H24" s="10"/>
       <c r="I24" s="10"/>
     </row>
-    <row r="25" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F25" s="9" t="s">
         <v>26</v>
       </c>
@@ -2455,7 +2458,7 @@
       <c r="H25" s="10"/>
       <c r="I25" s="10"/>
     </row>
-    <row r="26" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F26" s="9" t="s">
         <v>27</v>
       </c>
@@ -2463,7 +2466,7 @@
       <c r="H26" s="10"/>
       <c r="I26" s="10"/>
     </row>
-    <row r="27" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F27" s="9" t="s">
         <v>28</v>
       </c>
@@ -2471,7 +2474,7 @@
       <c r="H27" s="10"/>
       <c r="I27" s="10"/>
     </row>
-    <row r="28" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F28" s="9" t="s">
         <v>29</v>
       </c>
@@ -2482,7 +2485,7 @@
       </c>
       <c r="I28" s="12"/>
     </row>
-    <row r="29" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F29" s="9" t="s">
         <v>30</v>
       </c>
@@ -2490,7 +2493,7 @@
       <c r="H29" s="13"/>
       <c r="I29" s="13"/>
     </row>
-    <row r="30" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F30" s="9" t="s">
         <v>31</v>
       </c>
@@ -2501,8 +2504,8 @@
       </c>
       <c r="I30" s="12"/>
     </row>
-    <row r="31" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="32" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="11.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="32" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F32" s="9" t="s">
         <v>32</v>
       </c>
@@ -2510,7 +2513,7 @@
       <c r="H32" s="10"/>
       <c r="I32" s="10"/>
     </row>
-    <row r="33" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F33" s="9" t="s">
         <v>33</v>
       </c>
@@ -2518,7 +2521,7 @@
       <c r="H33" s="10"/>
       <c r="I33" s="10"/>
     </row>
-    <row r="34" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F34" s="9" t="s">
         <v>34</v>
       </c>
@@ -2526,7 +2529,7 @@
       <c r="H34" s="10"/>
       <c r="I34" s="10"/>
     </row>
-    <row r="35" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F35" s="9" t="s">
         <v>35</v>
       </c>
@@ -2534,7 +2537,7 @@
       <c r="H35" s="10"/>
       <c r="I35" s="10"/>
     </row>
-    <row r="36" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F36" s="9" t="s">
         <v>36</v>
       </c>
@@ -2542,7 +2545,7 @@
       <c r="H36" s="14"/>
       <c r="I36" s="14"/>
     </row>
-    <row r="37" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F37" s="9" t="s">
         <v>37</v>
       </c>
@@ -2553,7 +2556,7 @@
       </c>
       <c r="I37" s="12"/>
     </row>
-    <row r="38" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F38" s="9" t="s">
         <v>38</v>
       </c>
@@ -2564,7 +2567,7 @@
       </c>
       <c r="I38" s="12"/>
     </row>
-    <row r="39" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="15" t="s">
         <v>39</v>
       </c>
@@ -2581,7 +2584,7 @@
       </c>
       <c r="I39" s="12"/>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="16" t="s">
         <v>41</v>
       </c>
@@ -2595,7 +2598,7 @@
       <c r="H40" s="13"/>
       <c r="I40" s="13"/>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="16" t="s">
         <v>43</v>
       </c>
@@ -2612,7 +2615,8 @@
       </c>
       <c r="I41" s="12"/>
     </row>
-    <row r="43" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="43" customFormat="false" ht="32.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="9" t="s">
         <v>45</v>
       </c>
@@ -2627,7 +2631,8 @@
       <c r="H43" s="4"/>
       <c r="I43" s="4"/>
     </row>
-    <row r="45" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="45" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="18" t="s">
         <v>47</v>
       </c>
@@ -2640,7 +2645,7 @@
       <c r="H45" s="18"/>
       <c r="I45" s="18"/>
     </row>
-    <row r="46" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="18"/>
       <c r="B46" s="18"/>
       <c r="C46" s="18"/>
@@ -2651,7 +2656,7 @@
       <c r="H46" s="18"/>
       <c r="I46" s="18"/>
     </row>
-    <row r="47" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="18"/>
       <c r="B47" s="18"/>
       <c r="C47" s="18"/>
@@ -2662,7 +2667,8 @@
       <c r="H47" s="18"/>
       <c r="I47" s="18"/>
     </row>
-    <row r="49" customFormat="false" ht="11.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="49" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="19" t="s">
         <v>48</v>
       </c>
@@ -2751,9 +2757,9 @@
     <mergeCell ref="A45:I47"/>
     <mergeCell ref="A49:I49"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="true"/>
-  <pageMargins left="0.4" right="0.4" top="0.4" bottom="0.4" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.3" right="0.3" top="0.3" bottom="0.3" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>